<commit_message>
Updated files after submission of revised paper
</commit_message>
<xml_diff>
--- a/input_APWP.xlsx
+++ b/input_APWP.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bramvaes/Library/CloudStorage/GoogleDrive-bram.vaes@unimib.it/Other computers/My MacBook Pro/Python/TPW/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C740E8B-A384-A44D-A0AF-BFF5499CBCE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CA39A1D-9438-294A-8C37-835834478399}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-9560" yWindow="-21600" windowWidth="38400" windowHeight="21600" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-9560" yWindow="-21100" windowWidth="38400" windowHeight="21100" firstSheet="1" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="V23" sheetId="5" r:id="rId1"/>
@@ -18,6 +18,8 @@
     <sheet name="V23_int_5" sheetId="7" r:id="rId3"/>
     <sheet name="PWPs" sheetId="10" r:id="rId4"/>
     <sheet name="TPWPs" sheetId="8" r:id="rId5"/>
+    <sheet name="T12" sheetId="11" r:id="rId6"/>
+    <sheet name="M21" sheetId="14" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="18">
   <si>
     <t>lon</t>
   </si>
@@ -84,6 +86,12 @@
   <si>
     <t>lat_T08</t>
   </si>
+  <si>
+    <t>lon_D12_TPWP</t>
+  </si>
+  <si>
+    <t>lat_D12_TPWP</t>
+  </si>
 </sst>
 </file>
 
@@ -92,7 +100,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="20">
+  <fonts count="21">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -239,6 +247,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FF000000"/>
+      <name val="Courier New"/>
+      <family val="1"/>
     </font>
   </fonts>
   <fills count="33">
@@ -582,7 +596,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -604,6 +618,14 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -5223,10 +5245,14 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{29A839E9-DE8A-5B4F-BA37-1C653DA3C33D}">
-  <dimension ref="A1:J34"/>
+  <dimension ref="A1:L34"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <cols>
+    <col min="11" max="11" width="13.83203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.5" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:12">
       <c r="A1" s="4" t="s">
         <v>4</v>
       </c>
@@ -5257,8 +5283,14 @@
       <c r="J1" s="4" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="2" spans="1:10">
+      <c r="K1" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="L1" s="12" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12">
       <c r="A2" s="5">
         <v>0</v>
       </c>
@@ -5289,8 +5321,14 @@
       <c r="J2" s="3">
         <v>90</v>
       </c>
-    </row>
-    <row r="3" spans="1:10">
+      <c r="K2" s="3">
+        <v>173.9</v>
+      </c>
+      <c r="L2" s="3">
+        <v>88.5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12">
       <c r="A3" s="5">
         <v>1.18201219490578</v>
       </c>
@@ -5321,8 +5359,14 @@
       <c r="J3" s="3">
         <v>87.0682642268591</v>
       </c>
-    </row>
-    <row r="4" spans="1:10">
+      <c r="K3" s="3">
+        <v>146.73824099999999</v>
+      </c>
+      <c r="L3" s="3">
+        <v>86.865808000000001</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12">
       <c r="A4" s="5">
         <v>1.1743691358609101</v>
       </c>
@@ -5353,8 +5397,14 @@
       <c r="J4" s="3">
         <v>84.374368690408204</v>
       </c>
-    </row>
-    <row r="5" spans="1:10">
+      <c r="K4" s="3">
+        <v>144.67352500000001</v>
+      </c>
+      <c r="L4" s="3">
+        <v>84.375181999999995</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12">
       <c r="A5" s="5">
         <v>0.92054998461114701</v>
       </c>
@@ -5385,8 +5435,14 @@
       <c r="J5" s="3">
         <v>83.452106290388997</v>
       </c>
-    </row>
-    <row r="6" spans="1:10">
+      <c r="K5" s="3">
+        <v>137.11667800000001</v>
+      </c>
+      <c r="L5" s="3">
+        <v>83.313101000000003</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12">
       <c r="A6" s="5">
         <v>1.26892151026476</v>
       </c>
@@ -5417,8 +5473,14 @@
       <c r="J6" s="3">
         <v>83.075229039400796</v>
       </c>
-    </row>
-    <row r="7" spans="1:10">
+      <c r="K6" s="3">
+        <v>135.374943</v>
+      </c>
+      <c r="L6" s="3">
+        <v>82.526812000000007</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12">
       <c r="A7" s="5">
         <v>0.90834954750167796</v>
       </c>
@@ -5449,8 +5511,14 @@
       <c r="J7" s="3">
         <v>82.063469448681403</v>
       </c>
-    </row>
-    <row r="8" spans="1:10">
+      <c r="K7" s="3">
+        <v>173.50913</v>
+      </c>
+      <c r="L7" s="3">
+        <v>80.442550999999995</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12">
       <c r="A8" s="5">
         <v>0.80446278952633998</v>
       </c>
@@ -5481,8 +5549,14 @@
       <c r="J8" s="3">
         <v>81.405858545586597</v>
       </c>
-    </row>
-    <row r="9" spans="1:10">
+      <c r="K8" s="3">
+        <v>-168.53714500000001</v>
+      </c>
+      <c r="L8" s="3">
+        <v>78.015348000000003</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12">
       <c r="A9" s="5">
         <v>0.90975007803819197</v>
       </c>
@@ -5513,8 +5587,14 @@
       <c r="J9" s="3">
         <v>82.983224362435294</v>
       </c>
-    </row>
-    <row r="10" spans="1:10">
+      <c r="K9" s="3">
+        <v>-170.19886399999999</v>
+      </c>
+      <c r="L9" s="3">
+        <v>80.120726000000005</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12">
       <c r="A10" s="5">
         <v>1.2059772450903501</v>
       </c>
@@ -5545,8 +5625,14 @@
       <c r="J10" s="3">
         <v>86.681700671393202</v>
       </c>
-    </row>
-    <row r="11" spans="1:10">
+      <c r="K10" s="3">
+        <v>164.758837</v>
+      </c>
+      <c r="L10" s="3">
+        <v>82.687092000000007</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12">
       <c r="A11" s="5">
         <v>1.5025489247134101</v>
       </c>
@@ -5577,8 +5663,14 @@
       <c r="J11" s="3">
         <v>86.943856061572404</v>
       </c>
-    </row>
-    <row r="12" spans="1:10">
+      <c r="K11" s="3">
+        <v>154.02507900000001</v>
+      </c>
+      <c r="L11" s="3">
+        <v>84.875218000000004</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12">
       <c r="A12" s="5">
         <v>1.7916183110921799</v>
       </c>
@@ -5609,8 +5701,14 @@
       <c r="J12" s="3">
         <v>83.1402167177379</v>
       </c>
-    </row>
-    <row r="13" spans="1:10">
+      <c r="K12" s="3">
+        <v>145.046133</v>
+      </c>
+      <c r="L12" s="3">
+        <v>87.508296999999999</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12">
       <c r="A13" s="5">
         <v>1.3335158290931699</v>
       </c>
@@ -5641,8 +5739,14 @@
       <c r="J13" s="3">
         <v>81.694167236243104</v>
       </c>
-    </row>
-    <row r="14" spans="1:10">
+      <c r="K13" s="3">
+        <v>-82.387207000000004</v>
+      </c>
+      <c r="L13" s="3">
+        <v>81.954841999999999</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12">
       <c r="A14" s="5">
         <v>1.1101312603647699</v>
       </c>
@@ -5673,8 +5777,14 @@
       <c r="J14" s="3">
         <v>81.582270815839607</v>
       </c>
-    </row>
-    <row r="15" spans="1:10">
+      <c r="K14" s="3">
+        <v>-82.524327</v>
+      </c>
+      <c r="L14" s="3">
+        <v>78.684701000000004</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12">
       <c r="A15" s="5">
         <v>0.77272252658218199</v>
       </c>
@@ -5694,7 +5804,7 @@
         <v>78.988813532167995</v>
       </c>
     </row>
-    <row r="16" spans="1:10">
+    <row r="16" spans="1:12">
       <c r="A16" s="5">
         <v>1.2058040401502801</v>
       </c>
@@ -6077,4 +6187,1345 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76FEF3D4-8109-9B40-B708-7AAA5407ACA9}">
+  <dimension ref="A1:D34"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <cols>
+    <col min="1" max="4" width="10.83203125" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" s="9">
+        <v>353.9</v>
+      </c>
+      <c r="B2" s="9">
+        <v>-88.5</v>
+      </c>
+      <c r="C2" s="9">
+        <v>1.9</v>
+      </c>
+      <c r="D2" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" s="9">
+        <v>350</v>
+      </c>
+      <c r="B3" s="9">
+        <v>-86.6</v>
+      </c>
+      <c r="C3" s="9">
+        <v>1.8</v>
+      </c>
+      <c r="D3" s="2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" s="9">
+        <v>355.6</v>
+      </c>
+      <c r="B4" s="9">
+        <v>-84.2</v>
+      </c>
+      <c r="C4" s="9">
+        <v>2.6</v>
+      </c>
+      <c r="D4" s="2">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" s="9">
+        <v>0.3</v>
+      </c>
+      <c r="B5" s="9">
+        <v>-82.9</v>
+      </c>
+      <c r="C5" s="9">
+        <v>2.6</v>
+      </c>
+      <c r="D5" s="2">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" s="9">
+        <v>9</v>
+      </c>
+      <c r="B6" s="9">
+        <v>-80.5</v>
+      </c>
+      <c r="C6" s="9">
+        <v>2.9</v>
+      </c>
+      <c r="D6" s="2">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" s="9">
+        <v>25.6</v>
+      </c>
+      <c r="B7" s="9">
+        <v>-75.5</v>
+      </c>
+      <c r="C7" s="9">
+        <v>2.8</v>
+      </c>
+      <c r="D7" s="2">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
+      <c r="A8" s="9">
+        <v>35.299999999999997</v>
+      </c>
+      <c r="B8" s="9">
+        <v>-72.900000000000006</v>
+      </c>
+      <c r="C8" s="9">
+        <v>2.1</v>
+      </c>
+      <c r="D8" s="2">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
+      <c r="A9" s="9">
+        <v>43.3</v>
+      </c>
+      <c r="B9" s="9">
+        <v>-71.7</v>
+      </c>
+      <c r="C9" s="9">
+        <v>2.5</v>
+      </c>
+      <c r="D9" s="2">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
+      <c r="A10" s="9">
+        <v>49.2</v>
+      </c>
+      <c r="B10" s="9">
+        <v>-70.599999999999994</v>
+      </c>
+      <c r="C10" s="9">
+        <v>2.9</v>
+      </c>
+      <c r="D10" s="2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
+      <c r="A11" s="9">
+        <v>55.6</v>
+      </c>
+      <c r="B11" s="9">
+        <v>-69.400000000000006</v>
+      </c>
+      <c r="C11" s="9">
+        <v>2.5</v>
+      </c>
+      <c r="D11" s="2">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4">
+      <c r="A12" s="9">
+        <v>63.2</v>
+      </c>
+      <c r="B12" s="9">
+        <v>-67</v>
+      </c>
+      <c r="C12" s="9">
+        <v>3.3</v>
+      </c>
+      <c r="D12" s="2">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4">
+      <c r="A13" s="9">
+        <v>78.7</v>
+      </c>
+      <c r="B13" s="9">
+        <v>-58.2</v>
+      </c>
+      <c r="C13" s="9">
+        <v>3.3</v>
+      </c>
+      <c r="D13" s="2">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4">
+      <c r="A14" s="9">
+        <v>81.3</v>
+      </c>
+      <c r="B14" s="9">
+        <v>-53.6</v>
+      </c>
+      <c r="C14" s="9">
+        <v>2.6</v>
+      </c>
+      <c r="D14" s="2">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4">
+      <c r="A15" s="9">
+        <v>80.900000000000006</v>
+      </c>
+      <c r="B15" s="9">
+        <v>-49.3</v>
+      </c>
+      <c r="C15" s="9">
+        <v>2.8</v>
+      </c>
+      <c r="D15" s="2">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4">
+      <c r="A16" s="9">
+        <v>82.1</v>
+      </c>
+      <c r="B16" s="9">
+        <v>-45.8</v>
+      </c>
+      <c r="C16" s="9">
+        <v>6</v>
+      </c>
+      <c r="D16" s="2">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4">
+      <c r="A17" s="9">
+        <v>77.2</v>
+      </c>
+      <c r="B17" s="9">
+        <v>-53.1</v>
+      </c>
+      <c r="C17" s="9">
+        <v>6.4</v>
+      </c>
+      <c r="D17" s="2">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4">
+      <c r="A18" s="9">
+        <v>75.900000000000006</v>
+      </c>
+      <c r="B18" s="9">
+        <v>-55.4</v>
+      </c>
+      <c r="C18" s="9">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="D18" s="2">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4">
+      <c r="A19" s="9">
+        <v>73.900000000000006</v>
+      </c>
+      <c r="B19" s="9">
+        <v>-55.9</v>
+      </c>
+      <c r="C19" s="9">
+        <v>4.5999999999999996</v>
+      </c>
+      <c r="D19" s="2">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4">
+      <c r="A20" s="9">
+        <v>78.5</v>
+      </c>
+      <c r="B20" s="9">
+        <v>-62.1</v>
+      </c>
+      <c r="C20" s="9">
+        <v>3.4</v>
+      </c>
+      <c r="D20" s="2">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4">
+      <c r="A21" s="9">
+        <v>76.599999999999994</v>
+      </c>
+      <c r="B21" s="9">
+        <v>-66.8</v>
+      </c>
+      <c r="C21" s="9">
+        <v>2.9</v>
+      </c>
+      <c r="D21" s="2">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4">
+      <c r="A22" s="9">
+        <v>62.2</v>
+      </c>
+      <c r="B22" s="9">
+        <v>-69</v>
+      </c>
+      <c r="C22" s="9">
+        <v>2.8</v>
+      </c>
+      <c r="D22" s="2">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4">
+      <c r="A23" s="9">
+        <v>56.3</v>
+      </c>
+      <c r="B23" s="9">
+        <v>-64.599999999999994</v>
+      </c>
+      <c r="C23" s="9">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="D23" s="2">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4">
+      <c r="A24" s="9">
+        <v>50.4</v>
+      </c>
+      <c r="B24" s="9">
+        <v>-58.4</v>
+      </c>
+      <c r="C24" s="9">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="D24" s="2">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4">
+      <c r="A25" s="9">
+        <v>50</v>
+      </c>
+      <c r="B25" s="9">
+        <v>-53</v>
+      </c>
+      <c r="C25" s="9">
+        <v>2.5</v>
+      </c>
+      <c r="D25" s="2">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4">
+      <c r="A26" s="9">
+        <v>56.1</v>
+      </c>
+      <c r="B26" s="9">
+        <v>-48.3</v>
+      </c>
+      <c r="C26" s="9">
+        <v>3.6</v>
+      </c>
+      <c r="D26" s="2">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4">
+      <c r="A27" s="9">
+        <v>60.7</v>
+      </c>
+      <c r="B27" s="9">
+        <v>-44.7</v>
+      </c>
+      <c r="C27" s="9">
+        <v>3.6</v>
+      </c>
+      <c r="D27" s="2">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4">
+      <c r="A28" s="9">
+        <v>61.8</v>
+      </c>
+      <c r="B28" s="9">
+        <v>-44.3</v>
+      </c>
+      <c r="C28" s="9">
+        <v>2.6</v>
+      </c>
+      <c r="D28" s="2">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4">
+      <c r="A29" s="9">
+        <v>60.1</v>
+      </c>
+      <c r="B29" s="9">
+        <v>-39.799999999999997</v>
+      </c>
+      <c r="C29" s="9">
+        <v>2.9</v>
+      </c>
+      <c r="D29" s="2">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4">
+      <c r="A30" s="9">
+        <v>57.1</v>
+      </c>
+      <c r="B30" s="9">
+        <v>-34.4</v>
+      </c>
+      <c r="C30" s="9">
+        <v>2.8</v>
+      </c>
+      <c r="D30" s="2">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4">
+      <c r="A31" s="9">
+        <v>55.4</v>
+      </c>
+      <c r="B31" s="9">
+        <v>-32.9</v>
+      </c>
+      <c r="C31" s="9">
+        <v>2.4</v>
+      </c>
+      <c r="D31" s="2">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4">
+      <c r="A32" s="9">
+        <v>53.5</v>
+      </c>
+      <c r="B32" s="9">
+        <v>-31.3</v>
+      </c>
+      <c r="C32" s="9">
+        <v>2.8</v>
+      </c>
+      <c r="D32" s="2">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4">
+      <c r="A33" s="9">
+        <v>48.5</v>
+      </c>
+      <c r="B33" s="9">
+        <v>-28</v>
+      </c>
+      <c r="C33" s="9">
+        <v>3.9</v>
+      </c>
+      <c r="D33" s="2">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4">
+      <c r="A34" s="9">
+        <v>41.8</v>
+      </c>
+      <c r="B34" s="9">
+        <v>-25.1</v>
+      </c>
+      <c r="C34" s="9">
+        <v>4.9000000000000004</v>
+      </c>
+      <c r="D34" s="2">
+        <v>320</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F8BFA3E-B9AB-1444-8B50-D659ACC3D20D}">
+  <dimension ref="A1:G56"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <cols>
+    <col min="1" max="4" width="10.83203125" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" ht="19">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="G1" s="11"/>
+    </row>
+    <row r="2" spans="1:7" ht="19">
+      <c r="A2" s="10">
+        <v>0</v>
+      </c>
+      <c r="B2" s="10">
+        <v>-90</v>
+      </c>
+      <c r="C2" s="9">
+        <v>1.9</v>
+      </c>
+      <c r="D2" s="2">
+        <v>0</v>
+      </c>
+      <c r="G2" s="11"/>
+    </row>
+    <row r="3" spans="1:7" ht="19">
+      <c r="A3" s="10">
+        <v>7.1899999999999897</v>
+      </c>
+      <c r="B3" s="10">
+        <v>-84.69</v>
+      </c>
+      <c r="C3" s="9">
+        <v>1.9</v>
+      </c>
+      <c r="D3" s="2">
+        <v>10</v>
+      </c>
+      <c r="G3" s="11"/>
+    </row>
+    <row r="4" spans="1:7" ht="19">
+      <c r="A4" s="10">
+        <v>1.92</v>
+      </c>
+      <c r="B4" s="10">
+        <v>-83.29</v>
+      </c>
+      <c r="C4" s="9">
+        <v>2</v>
+      </c>
+      <c r="D4" s="2">
+        <v>20</v>
+      </c>
+      <c r="G4" s="11"/>
+    </row>
+    <row r="5" spans="1:7" ht="19">
+      <c r="A5" s="10">
+        <v>12.079999999999901</v>
+      </c>
+      <c r="B5" s="10">
+        <v>-81.459999999999994</v>
+      </c>
+      <c r="C5" s="9">
+        <v>2.4</v>
+      </c>
+      <c r="D5" s="2">
+        <v>30</v>
+      </c>
+      <c r="G5" s="11"/>
+    </row>
+    <row r="6" spans="1:7" ht="19">
+      <c r="A6" s="10">
+        <v>27.3399999999999</v>
+      </c>
+      <c r="B6" s="10">
+        <v>-76.27</v>
+      </c>
+      <c r="C6" s="9">
+        <v>3</v>
+      </c>
+      <c r="D6" s="2">
+        <v>40</v>
+      </c>
+      <c r="G6" s="11"/>
+    </row>
+    <row r="7" spans="1:7" ht="19">
+      <c r="A7" s="10">
+        <v>34.389999999999901</v>
+      </c>
+      <c r="B7" s="10">
+        <v>-74.729999999999905</v>
+      </c>
+      <c r="C7" s="9">
+        <v>2.8</v>
+      </c>
+      <c r="D7" s="2">
+        <v>50</v>
+      </c>
+      <c r="G7" s="11"/>
+    </row>
+    <row r="8" spans="1:7" ht="19">
+      <c r="A8" s="10">
+        <v>39.74</v>
+      </c>
+      <c r="B8" s="10">
+        <v>-73.17</v>
+      </c>
+      <c r="C8" s="9">
+        <v>2.6</v>
+      </c>
+      <c r="D8" s="2">
+        <v>60</v>
+      </c>
+      <c r="G8" s="11"/>
+    </row>
+    <row r="9" spans="1:7" ht="19">
+      <c r="A9" s="10">
+        <v>48.559999999999903</v>
+      </c>
+      <c r="B9" s="10">
+        <v>-71.09</v>
+      </c>
+      <c r="C9" s="9">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="D9" s="2">
+        <v>70</v>
+      </c>
+      <c r="G9" s="11"/>
+    </row>
+    <row r="10" spans="1:7" ht="19">
+      <c r="A10" s="10">
+        <v>52.15</v>
+      </c>
+      <c r="B10" s="10">
+        <v>-70.23</v>
+      </c>
+      <c r="C10" s="9">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="D10" s="2">
+        <v>80</v>
+      </c>
+      <c r="G10" s="11"/>
+    </row>
+    <row r="11" spans="1:7" ht="19">
+      <c r="A11" s="10">
+        <v>61.229999999999897</v>
+      </c>
+      <c r="B11" s="10">
+        <v>-69.260000000000005</v>
+      </c>
+      <c r="C11" s="9">
+        <v>2.4</v>
+      </c>
+      <c r="D11" s="2">
+        <v>90</v>
+      </c>
+      <c r="G11" s="11"/>
+    </row>
+    <row r="12" spans="1:7" ht="19">
+      <c r="A12" s="10">
+        <v>69.699999999999903</v>
+      </c>
+      <c r="B12" s="10">
+        <v>-66.08</v>
+      </c>
+      <c r="C12" s="9">
+        <v>2.6</v>
+      </c>
+      <c r="D12" s="2">
+        <v>100</v>
+      </c>
+      <c r="G12" s="11"/>
+    </row>
+    <row r="13" spans="1:7" ht="19">
+      <c r="A13" s="10">
+        <v>75.430000000000007</v>
+      </c>
+      <c r="B13" s="10">
+        <v>-61.26</v>
+      </c>
+      <c r="C13" s="9">
+        <v>3.4</v>
+      </c>
+      <c r="D13" s="2">
+        <v>110</v>
+      </c>
+      <c r="G13" s="11"/>
+    </row>
+    <row r="14" spans="1:7" ht="19">
+      <c r="A14" s="10">
+        <v>79.279999999999902</v>
+      </c>
+      <c r="B14" s="10">
+        <v>-57.31</v>
+      </c>
+      <c r="C14" s="9">
+        <v>3.4</v>
+      </c>
+      <c r="D14" s="2">
+        <v>120</v>
+      </c>
+      <c r="G14" s="11"/>
+    </row>
+    <row r="15" spans="1:7" ht="19">
+      <c r="A15" s="10">
+        <v>78.729999999999905</v>
+      </c>
+      <c r="B15" s="10">
+        <v>-54.21</v>
+      </c>
+      <c r="C15" s="9">
+        <v>3.9</v>
+      </c>
+      <c r="D15" s="2">
+        <v>130</v>
+      </c>
+      <c r="G15" s="11"/>
+    </row>
+    <row r="16" spans="1:7" ht="19">
+      <c r="A16" s="10">
+        <v>78.239999999999995</v>
+      </c>
+      <c r="B16" s="10">
+        <v>-50.7</v>
+      </c>
+      <c r="C16" s="9">
+        <v>4</v>
+      </c>
+      <c r="D16" s="2">
+        <v>140</v>
+      </c>
+      <c r="G16" s="11"/>
+    </row>
+    <row r="17" spans="1:7" ht="19">
+      <c r="A17" s="10">
+        <v>76.55</v>
+      </c>
+      <c r="B17" s="10">
+        <v>-48.11</v>
+      </c>
+      <c r="C17" s="9">
+        <v>4.2</v>
+      </c>
+      <c r="D17" s="2">
+        <v>150</v>
+      </c>
+      <c r="G17" s="11"/>
+    </row>
+    <row r="18" spans="1:7" ht="19">
+      <c r="A18" s="10">
+        <v>75.219999999999899</v>
+      </c>
+      <c r="B18" s="10">
+        <v>-54.27</v>
+      </c>
+      <c r="C18" s="9">
+        <v>4</v>
+      </c>
+      <c r="D18" s="2">
+        <v>160</v>
+      </c>
+      <c r="G18" s="11"/>
+    </row>
+    <row r="19" spans="1:7" ht="19">
+      <c r="A19" s="10">
+        <v>74.809999999999903</v>
+      </c>
+      <c r="B19" s="10">
+        <v>-56.37</v>
+      </c>
+      <c r="C19" s="9">
+        <v>3.8</v>
+      </c>
+      <c r="D19" s="2">
+        <v>170</v>
+      </c>
+      <c r="G19" s="11"/>
+    </row>
+    <row r="20" spans="1:7" ht="19">
+      <c r="A20" s="10">
+        <v>71.569999999999993</v>
+      </c>
+      <c r="B20" s="10">
+        <v>-60.79</v>
+      </c>
+      <c r="C20" s="9">
+        <v>3.3</v>
+      </c>
+      <c r="D20" s="2">
+        <v>180</v>
+      </c>
+      <c r="G20" s="11"/>
+    </row>
+    <row r="21" spans="1:7" ht="19">
+      <c r="A21" s="10">
+        <v>66.989999999999995</v>
+      </c>
+      <c r="B21" s="10">
+        <v>-63.44</v>
+      </c>
+      <c r="C21" s="9">
+        <v>2.6</v>
+      </c>
+      <c r="D21" s="2">
+        <v>190</v>
+      </c>
+      <c r="G21" s="11"/>
+    </row>
+    <row r="22" spans="1:7" ht="19">
+      <c r="A22" s="10">
+        <v>62.699999999999903</v>
+      </c>
+      <c r="B22" s="10">
+        <v>-63.87</v>
+      </c>
+      <c r="C22" s="9">
+        <v>2.5</v>
+      </c>
+      <c r="D22" s="2">
+        <v>200</v>
+      </c>
+      <c r="G22" s="11"/>
+    </row>
+    <row r="23" spans="1:7" ht="19">
+      <c r="A23" s="10">
+        <v>57.259999999999899</v>
+      </c>
+      <c r="B23" s="10">
+        <v>-63.18</v>
+      </c>
+      <c r="C23" s="9">
+        <v>2.5</v>
+      </c>
+      <c r="D23" s="2">
+        <v>210</v>
+      </c>
+      <c r="G23" s="11"/>
+    </row>
+    <row r="24" spans="1:7" ht="19">
+      <c r="A24" s="10">
+        <v>56.59</v>
+      </c>
+      <c r="B24" s="10">
+        <v>-60.47</v>
+      </c>
+      <c r="C24" s="9">
+        <v>2.8</v>
+      </c>
+      <c r="D24" s="2">
+        <v>220</v>
+      </c>
+      <c r="G24" s="11"/>
+    </row>
+    <row r="25" spans="1:7" ht="19">
+      <c r="A25" s="10">
+        <v>58.459999999999901</v>
+      </c>
+      <c r="B25" s="10">
+        <v>-52.79</v>
+      </c>
+      <c r="C25" s="9">
+        <v>3.4</v>
+      </c>
+      <c r="D25" s="2">
+        <v>230</v>
+      </c>
+      <c r="G25" s="11"/>
+    </row>
+    <row r="26" spans="1:7" ht="19">
+      <c r="A26" s="10">
+        <v>60.419999999999902</v>
+      </c>
+      <c r="B26" s="10">
+        <v>-47.18</v>
+      </c>
+      <c r="C26" s="9">
+        <v>3.5</v>
+      </c>
+      <c r="D26" s="2">
+        <v>240</v>
+      </c>
+      <c r="G26" s="11"/>
+    </row>
+    <row r="27" spans="1:7" ht="19">
+      <c r="A27" s="10">
+        <v>62.87</v>
+      </c>
+      <c r="B27" s="10">
+        <v>-42.64</v>
+      </c>
+      <c r="C27" s="9">
+        <v>4</v>
+      </c>
+      <c r="D27" s="2">
+        <v>250</v>
+      </c>
+      <c r="G27" s="11"/>
+    </row>
+    <row r="28" spans="1:7" ht="19">
+      <c r="A28" s="10">
+        <v>62.549999999999898</v>
+      </c>
+      <c r="B28" s="10">
+        <v>-38.57</v>
+      </c>
+      <c r="C28" s="9">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="D28" s="2">
+        <v>260</v>
+      </c>
+      <c r="G28" s="11"/>
+    </row>
+    <row r="29" spans="1:7" ht="19">
+      <c r="A29" s="10">
+        <v>60.949999999999903</v>
+      </c>
+      <c r="B29" s="10">
+        <v>-38.64</v>
+      </c>
+      <c r="C29" s="9">
+        <v>4.7</v>
+      </c>
+      <c r="D29" s="2">
+        <v>270</v>
+      </c>
+      <c r="G29" s="11"/>
+    </row>
+    <row r="30" spans="1:7" ht="19">
+      <c r="A30" s="10">
+        <v>58.21</v>
+      </c>
+      <c r="B30" s="10">
+        <v>-36.029999999999902</v>
+      </c>
+      <c r="C30" s="9">
+        <v>5.3</v>
+      </c>
+      <c r="D30" s="2">
+        <v>280</v>
+      </c>
+      <c r="G30" s="11"/>
+    </row>
+    <row r="31" spans="1:7" ht="19">
+      <c r="A31" s="10">
+        <v>55.229999999999897</v>
+      </c>
+      <c r="B31" s="10">
+        <v>-32.06</v>
+      </c>
+      <c r="C31" s="9">
+        <v>5.4</v>
+      </c>
+      <c r="D31" s="2">
+        <v>290</v>
+      </c>
+      <c r="G31" s="11"/>
+    </row>
+    <row r="32" spans="1:7" ht="19">
+      <c r="A32" s="10">
+        <v>51.979999999999897</v>
+      </c>
+      <c r="B32" s="10">
+        <v>-32.130000000000003</v>
+      </c>
+      <c r="C32" s="9">
+        <v>5</v>
+      </c>
+      <c r="D32" s="2">
+        <v>300</v>
+      </c>
+      <c r="G32" s="11"/>
+    </row>
+    <row r="33" spans="1:7" ht="19">
+      <c r="A33" s="10">
+        <v>50.569999999999901</v>
+      </c>
+      <c r="B33" s="10">
+        <v>-31.3399999999999</v>
+      </c>
+      <c r="C33" s="9">
+        <v>5.7</v>
+      </c>
+      <c r="D33" s="2">
+        <v>310</v>
+      </c>
+      <c r="G33" s="11"/>
+    </row>
+    <row r="34" spans="1:7" ht="19">
+      <c r="A34" s="10">
+        <v>49.459999999999901</v>
+      </c>
+      <c r="B34" s="10">
+        <v>-26.329999999999899</v>
+      </c>
+      <c r="C34" s="9">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="D34" s="2">
+        <v>320</v>
+      </c>
+      <c r="G34" s="11"/>
+    </row>
+    <row r="35" spans="1:7" ht="19">
+      <c r="A35" s="10">
+        <v>47.91</v>
+      </c>
+      <c r="B35" s="10">
+        <v>-23.909999999999997</v>
+      </c>
+      <c r="C35" s="9">
+        <v>0</v>
+      </c>
+      <c r="D35" s="2">
+        <v>330</v>
+      </c>
+      <c r="G35" s="11"/>
+    </row>
+    <row r="36" spans="1:7" ht="19">
+      <c r="A36" s="10">
+        <v>38.47</v>
+      </c>
+      <c r="B36" s="10">
+        <v>-19.099999999999994</v>
+      </c>
+      <c r="C36" s="9">
+        <v>0</v>
+      </c>
+      <c r="D36" s="2">
+        <v>340</v>
+      </c>
+      <c r="G36" s="11"/>
+    </row>
+    <row r="37" spans="1:7" ht="19">
+      <c r="A37" s="10">
+        <v>26.379999999999995</v>
+      </c>
+      <c r="B37" s="10">
+        <v>-11.519999999999996</v>
+      </c>
+      <c r="C37" s="9">
+        <v>0</v>
+      </c>
+      <c r="D37" s="2">
+        <v>350</v>
+      </c>
+      <c r="G37" s="11"/>
+    </row>
+    <row r="38" spans="1:7" ht="19">
+      <c r="A38" s="10">
+        <v>20.03</v>
+      </c>
+      <c r="B38" s="10">
+        <v>-6.3199999999999932</v>
+      </c>
+      <c r="C38" s="9">
+        <v>0</v>
+      </c>
+      <c r="D38" s="2">
+        <v>360</v>
+      </c>
+      <c r="G38" s="11"/>
+    </row>
+    <row r="39" spans="1:7" ht="19">
+      <c r="A39" s="10">
+        <v>18.079999999999998</v>
+      </c>
+      <c r="B39" s="10">
+        <v>-4.6099999999999994</v>
+      </c>
+      <c r="C39" s="9">
+        <v>0</v>
+      </c>
+      <c r="D39" s="2">
+        <v>370</v>
+      </c>
+      <c r="G39" s="11"/>
+    </row>
+    <row r="40" spans="1:7" ht="19">
+      <c r="A40" s="10">
+        <v>17.560000000000002</v>
+      </c>
+      <c r="B40" s="10">
+        <v>-3.9699999999999989</v>
+      </c>
+      <c r="C40" s="9">
+        <v>0</v>
+      </c>
+      <c r="D40" s="2">
+        <v>380</v>
+      </c>
+      <c r="G40" s="11"/>
+    </row>
+    <row r="41" spans="1:7" ht="19">
+      <c r="A41" s="10">
+        <v>16.379999999999995</v>
+      </c>
+      <c r="B41" s="10">
+        <v>-9.769999999999996</v>
+      </c>
+      <c r="C41" s="9">
+        <v>0</v>
+      </c>
+      <c r="D41" s="2">
+        <v>390</v>
+      </c>
+      <c r="G41" s="11"/>
+    </row>
+    <row r="42" spans="1:7" ht="19">
+      <c r="A42" s="10">
+        <v>13.549999999999997</v>
+      </c>
+      <c r="B42" s="10">
+        <v>-7.9200000000000017</v>
+      </c>
+      <c r="C42" s="9">
+        <v>0</v>
+      </c>
+      <c r="D42" s="2">
+        <v>400</v>
+      </c>
+      <c r="G42" s="11"/>
+    </row>
+    <row r="43" spans="1:7" ht="19">
+      <c r="A43" s="10">
+        <v>13.950000000000003</v>
+      </c>
+      <c r="B43" s="10">
+        <v>-21.689999999999998</v>
+      </c>
+      <c r="C43" s="9">
+        <v>0</v>
+      </c>
+      <c r="D43" s="2">
+        <v>410</v>
+      </c>
+      <c r="G43" s="11"/>
+    </row>
+    <row r="44" spans="1:7" ht="19">
+      <c r="A44" s="10">
+        <v>5.0049999999999955</v>
+      </c>
+      <c r="B44" s="10">
+        <v>-4.5998000000000019</v>
+      </c>
+      <c r="C44" s="9">
+        <v>0</v>
+      </c>
+      <c r="D44" s="2">
+        <v>420</v>
+      </c>
+      <c r="G44" s="11"/>
+    </row>
+    <row r="45" spans="1:7" ht="19">
+      <c r="A45" s="10">
+        <v>-1.3777000000000044</v>
+      </c>
+      <c r="B45" s="10">
+        <v>13.486999999999995</v>
+      </c>
+      <c r="C45" s="9">
+        <v>0</v>
+      </c>
+      <c r="D45" s="2">
+        <v>430</v>
+      </c>
+      <c r="G45" s="11"/>
+    </row>
+    <row r="46" spans="1:7" ht="19">
+      <c r="A46" s="10">
+        <v>-6.3199999999999932</v>
+      </c>
+      <c r="B46" s="10">
+        <v>32.11</v>
+      </c>
+      <c r="C46" s="9">
+        <v>0</v>
+      </c>
+      <c r="D46" s="2">
+        <v>440</v>
+      </c>
+      <c r="G46" s="11"/>
+    </row>
+    <row r="47" spans="1:7" ht="19">
+      <c r="A47" s="10">
+        <v>-1</v>
+      </c>
+      <c r="B47" s="10">
+        <v>36</v>
+      </c>
+      <c r="C47" s="9">
+        <v>0</v>
+      </c>
+      <c r="D47" s="2">
+        <v>450</v>
+      </c>
+      <c r="G47" s="11"/>
+    </row>
+    <row r="48" spans="1:7" ht="19">
+      <c r="A48" s="10">
+        <v>3.0600000000000023</v>
+      </c>
+      <c r="B48" s="10">
+        <v>34.89</v>
+      </c>
+      <c r="C48" s="9">
+        <v>0</v>
+      </c>
+      <c r="D48" s="2">
+        <v>460</v>
+      </c>
+      <c r="G48" s="11"/>
+    </row>
+    <row r="49" spans="1:7" ht="19">
+      <c r="A49" s="10">
+        <v>4.9599999999999937</v>
+      </c>
+      <c r="B49" s="10">
+        <v>34.799999999999997</v>
+      </c>
+      <c r="C49" s="9">
+        <v>0</v>
+      </c>
+      <c r="D49" s="2">
+        <v>470</v>
+      </c>
+      <c r="G49" s="11"/>
+    </row>
+    <row r="50" spans="1:7" ht="19">
+      <c r="A50" s="10">
+        <v>7.7099999999999937</v>
+      </c>
+      <c r="B50" s="10">
+        <v>30.83</v>
+      </c>
+      <c r="C50" s="9">
+        <v>0</v>
+      </c>
+      <c r="D50" s="2">
+        <v>480</v>
+      </c>
+      <c r="G50" s="11"/>
+    </row>
+    <row r="51" spans="1:7" ht="19">
+      <c r="A51" s="10">
+        <v>9.1500000000000057</v>
+      </c>
+      <c r="B51" s="10">
+        <v>27.75</v>
+      </c>
+      <c r="C51" s="9">
+        <v>0</v>
+      </c>
+      <c r="D51" s="2">
+        <v>490</v>
+      </c>
+      <c r="G51" s="11"/>
+    </row>
+    <row r="52" spans="1:7" ht="19">
+      <c r="A52" s="10">
+        <v>11.030000000000001</v>
+      </c>
+      <c r="B52" s="10">
+        <v>24</v>
+      </c>
+      <c r="C52" s="9">
+        <v>0</v>
+      </c>
+      <c r="D52" s="2">
+        <v>500</v>
+      </c>
+      <c r="G52" s="11"/>
+    </row>
+    <row r="53" spans="1:7" ht="19">
+      <c r="A53" s="10">
+        <v>10.459999999999994</v>
+      </c>
+      <c r="B53" s="10">
+        <v>22.019999999999996</v>
+      </c>
+      <c r="C53" s="9">
+        <v>0</v>
+      </c>
+      <c r="D53" s="2">
+        <v>510</v>
+      </c>
+      <c r="G53" s="11"/>
+    </row>
+    <row r="54" spans="1:7" ht="19">
+      <c r="A54" s="10">
+        <v>4.8499999999999943</v>
+      </c>
+      <c r="B54" s="10">
+        <v>19.959999999999994</v>
+      </c>
+      <c r="C54" s="9">
+        <v>0</v>
+      </c>
+      <c r="D54" s="2">
+        <v>520</v>
+      </c>
+      <c r="G54" s="11"/>
+    </row>
+    <row r="55" spans="1:7" ht="19">
+      <c r="A55" s="10">
+        <v>-0.78000000000000114</v>
+      </c>
+      <c r="B55" s="10">
+        <v>15.019999999999996</v>
+      </c>
+      <c r="C55" s="9">
+        <v>0</v>
+      </c>
+      <c r="D55" s="2">
+        <v>530</v>
+      </c>
+      <c r="G55" s="11"/>
+    </row>
+    <row r="56" spans="1:7">
+      <c r="A56" s="10">
+        <v>-2.1599999999999966</v>
+      </c>
+      <c r="B56" s="10">
+        <v>10.450000000000003</v>
+      </c>
+      <c r="C56" s="9">
+        <v>0</v>
+      </c>
+      <c r="D56" s="2">
+        <v>540</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>